<commit_message>
feat(points): make Part C optional with complete output before points extraction
Reorder workflow so output files (3-tab xlsx, sitemodel.json, manifest.json)
are written immediately after Part B extraction. Part C (points extraction)
becomes an optional follow-up that updates existing files in-place (4-tab xlsx).

- Swap Steps 6/7 in SKILL.md: OUTPUT before POINTS
- Add equipment graphics navigation guidance to points-extraction.md
- Add two-phase output documentation to output-format.md
- Add points_list tab support to write_xlsx.py
- Add points extraction hints to bms-ui-patterns.md
- Update CLAUDE.md workflow description

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/final_output.xlsx
+++ b/examples/final_output.xlsx
@@ -1,19 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="27815"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/howardmann/Work/cim_github/bms-extractor/examples/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="760" windowWidth="28800" windowHeight="17500" tabRatio="500" activeTab="2"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="levels_and_zones" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="equipment_list" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="equipment_types" sheetId="3" r:id="rId7"/>
+    <sheet name="levels_and_zones" sheetId="1" r:id="rId1"/>
+    <sheet name="equipment_list" sheetId="2" r:id="rId2"/>
+    <sheet name="points_list" sheetId="4" r:id="rId3"/>
+    <sheet name="equipment_types" sheetId="3" r:id="rId4"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0" concurrentCalc="0"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{79F54976-1DA5-4618-B147-4CDE4B953A38}">
+      <x14:workbookPr defaultImageDpi="32767"/>
+    </ext>
+    <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{7523E5D3-25F3-A5E0-1632-64F254C22452}">
+      <mx:ArchID Flags="2"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1066" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1347" uniqueCount="303">
   <si>
     <t>level</t>
   </si>
@@ -655,37 +672,317 @@
   </si>
   <si>
     <t>Zones</t>
+  </si>
+  <si>
+    <t>HR-Centre</t>
+  </si>
+  <si>
+    <t>AHAC (L1–L5)</t>
+  </si>
+  <si>
+    <t>Off</t>
+  </si>
+  <si>
+    <t>AHAC</t>
+  </si>
+  <si>
+    <t>Call To Start</t>
+  </si>
+  <si>
+    <t>CallToStart</t>
+  </si>
+  <si>
+    <t>CHW Valve Signal</t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t>CHW_Valve</t>
+  </si>
+  <si>
+    <t>CHWV</t>
+  </si>
+  <si>
+    <t>Controls Enabled</t>
+  </si>
+  <si>
+    <t>Disabled</t>
+  </si>
+  <si>
+    <t>ControlsEnabled</t>
+  </si>
+  <si>
+    <t>Economy Dampers</t>
+  </si>
+  <si>
+    <t>Economy_Damper_ToScreen</t>
+  </si>
+  <si>
+    <t>Economy Mode</t>
+  </si>
+  <si>
+    <t>Economy_Mode_Enabled</t>
+  </si>
+  <si>
+    <t>Fan Run On Time</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>RunOnTime</t>
+  </si>
+  <si>
+    <t>Filters</t>
+  </si>
+  <si>
+    <t>Clean</t>
+  </si>
+  <si>
+    <t>Filter_Status</t>
+  </si>
+  <si>
+    <t>In Auto</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>(no DOM binding)</t>
+  </si>
+  <si>
+    <t>O/A Damper</t>
+  </si>
+  <si>
+    <t>OA_Damper</t>
+  </si>
+  <si>
+    <t>O/S (L1–L5)</t>
+  </si>
+  <si>
+    <t>Opt_Start</t>
+  </si>
+  <si>
+    <t>OAH</t>
+  </si>
+  <si>
+    <t>%RH</t>
+  </si>
+  <si>
+    <t>OAT</t>
+  </si>
+  <si>
+    <t>°C</t>
+  </si>
+  <si>
+    <t>Out Of Service</t>
+  </si>
+  <si>
+    <t>R/A Damper</t>
+  </si>
+  <si>
+    <t>RA_Damper</t>
+  </si>
+  <si>
+    <t>R/A Duct Pressure</t>
+  </si>
+  <si>
+    <t>Pa</t>
+  </si>
+  <si>
+    <t>RA_StaticPressure</t>
+  </si>
+  <si>
+    <t>R/A Pressure Setpoint</t>
+  </si>
+  <si>
+    <t>RA_DuctPressSPT</t>
+  </si>
+  <si>
+    <t>RAF Alarm</t>
+  </si>
+  <si>
+    <t>Normal</t>
+  </si>
+  <si>
+    <t>RAF_Alarm</t>
+  </si>
+  <si>
+    <t>RAF Call</t>
+  </si>
+  <si>
+    <t>RAF_Call</t>
+  </si>
+  <si>
+    <t>RAF HLI Auto/Hand</t>
+  </si>
+  <si>
+    <t>Auto</t>
+  </si>
+  <si>
+    <t>HLI_HAND_AUTO</t>
+  </si>
+  <si>
+    <t>RAF HLI Frequency</t>
+  </si>
+  <si>
+    <t>Hz</t>
+  </si>
+  <si>
+    <t>HLI_Freq</t>
+  </si>
+  <si>
+    <t>RAF Speed</t>
+  </si>
+  <si>
+    <t>RAF_Speed</t>
+  </si>
+  <si>
+    <t>RAF Status</t>
+  </si>
+  <si>
+    <t>Stopped</t>
+  </si>
+  <si>
+    <t>RAF_Status</t>
+  </si>
+  <si>
+    <t>Relief Damper</t>
+  </si>
+  <si>
+    <t>Relief_Damper</t>
+  </si>
+  <si>
+    <t>Return Air Humidity</t>
+  </si>
+  <si>
+    <t>Common_RAH</t>
+  </si>
+  <si>
+    <t>Return Air Temp</t>
+  </si>
+  <si>
+    <t>Common_RAT</t>
+  </si>
+  <si>
+    <t>S/A Duct Pressure</t>
+  </si>
+  <si>
+    <t>SA_StaticPressure</t>
+  </si>
+  <si>
+    <t>S/A Pressure Setpoint</t>
+  </si>
+  <si>
+    <t>SA_DuctPressSPT</t>
+  </si>
+  <si>
+    <t>SAF Alarm</t>
+  </si>
+  <si>
+    <t>SAF_Alarm</t>
+  </si>
+  <si>
+    <t>SAF Call</t>
+  </si>
+  <si>
+    <t>SAF_Call</t>
+  </si>
+  <si>
+    <t>SAF HLI Auto/Hand</t>
+  </si>
+  <si>
+    <t>SAF HLI Frequency</t>
+  </si>
+  <si>
+    <t>SAF Speed</t>
+  </si>
+  <si>
+    <t>SAF_Speed</t>
+  </si>
+  <si>
+    <t>SAF Status</t>
+  </si>
+  <si>
+    <t>SAF_Status</t>
+  </si>
+  <si>
+    <t>SAT</t>
+  </si>
+  <si>
+    <t>Schedule (L1–L5)</t>
+  </si>
+  <si>
+    <t>Schedule</t>
+  </si>
+  <si>
+    <t>Selected VAV Offset</t>
+  </si>
+  <si>
+    <t>ZoneOffset</t>
+  </si>
+  <si>
+    <t>Supply Temp Setpoint</t>
+  </si>
+  <si>
+    <t>SupplyTempSPT</t>
+  </si>
+  <si>
+    <t>graphic_point_name</t>
+  </si>
+  <si>
+    <t>graphic_value</t>
+  </si>
+  <si>
+    <t>graphic_unit</t>
+  </si>
+  <si>
+    <t>underlying_point_name</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="5">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -693,50 +990,49 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="9">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium7"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -744,7 +1040,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -934,21 +1230,24 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr enableFormatConditionsCalculation="0">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:Z18"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="67.13"/>
-    <col customWidth="1" min="3" max="3" width="42.38"/>
+    <col min="2" max="2" width="67.1640625" customWidth="1"/>
+    <col min="3" max="3" width="42.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -984,7 +1283,7 @@
       <c r="Y1" s="2"/>
       <c r="Z1" s="2"/>
     </row>
-    <row r="2">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -998,7 +1297,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
@@ -1012,7 +1311,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A4" s="3" t="s">
         <v>11</v>
       </c>
@@ -1026,7 +1325,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A5" s="3" t="s">
         <v>15</v>
       </c>
@@ -1040,7 +1339,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A6" s="3" t="s">
         <v>19</v>
       </c>
@@ -1054,7 +1353,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A7" s="3" t="s">
         <v>21</v>
       </c>
@@ -1068,7 +1367,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A8" s="3" t="s">
         <v>23</v>
       </c>
@@ -1082,7 +1381,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A9" s="3" t="s">
         <v>25</v>
       </c>
@@ -1096,7 +1395,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A10" s="3" t="s">
         <v>29</v>
       </c>
@@ -1110,7 +1409,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A11" s="3" t="s">
         <v>31</v>
       </c>
@@ -1124,7 +1423,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>33</v>
       </c>
@@ -1138,7 +1437,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>35</v>
       </c>
@@ -1152,7 +1451,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>39</v>
       </c>
@@ -1166,7 +1465,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>43</v>
       </c>
@@ -1180,7 +1479,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>45</v>
       </c>
@@ -1194,7 +1493,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>49</v>
       </c>
@@ -1202,7 +1501,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.15">
       <c r="A18" s="3" t="s">
         <v>50</v>
       </c>
@@ -1212,38 +1511,40 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="D3"/>
-    <hyperlink r:id="rId2" ref="D4"/>
-    <hyperlink r:id="rId3" ref="D5"/>
-    <hyperlink r:id="rId4" ref="D6"/>
-    <hyperlink r:id="rId5" ref="D7"/>
-    <hyperlink r:id="rId6" ref="D8"/>
-    <hyperlink r:id="rId7" ref="D9"/>
-    <hyperlink r:id="rId8" ref="D10"/>
-    <hyperlink r:id="rId9" ref="D11"/>
-    <hyperlink r:id="rId10" ref="D12"/>
-    <hyperlink r:id="rId11" ref="D13"/>
-    <hyperlink r:id="rId12" ref="D14"/>
-    <hyperlink r:id="rId13" ref="D15"/>
-    <hyperlink r:id="rId14" ref="D16"/>
+    <hyperlink ref="D3" r:id="rId1"/>
+    <hyperlink ref="D4" r:id="rId2"/>
+    <hyperlink ref="D5" r:id="rId3"/>
+    <hyperlink ref="D6" r:id="rId4"/>
+    <hyperlink ref="D7" r:id="rId5"/>
+    <hyperlink ref="D8" r:id="rId6"/>
+    <hyperlink ref="D9" r:id="rId7"/>
+    <hyperlink ref="D10" r:id="rId8"/>
+    <hyperlink ref="D11" r:id="rId9"/>
+    <hyperlink ref="D12" r:id="rId10"/>
+    <hyperlink ref="D13" r:id="rId11"/>
+    <hyperlink ref="D14" r:id="rId12"/>
+    <hyperlink ref="D15" r:id="rId13"/>
+    <hyperlink ref="D16" r:id="rId14"/>
   </hyperlinks>
-  <drawing r:id="rId15"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr enableFormatConditionsCalculation="0">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:Z184"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="20.75"/>
-    <col customWidth="1" min="3" max="3" width="24.5"/>
-    <col customWidth="1" min="4" max="4" width="24.88"/>
+    <col min="1" max="1" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.6640625" customWidth="1"/>
+    <col min="3" max="3" width="24.5" customWidth="1"/>
+    <col min="4" max="4" width="24.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>51</v>
       </c>
@@ -1281,7 +1582,7 @@
       <c r="Y1" s="2"/>
       <c r="Z1" s="2"/>
     </row>
-    <row r="2">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A2" s="3" t="s">
         <v>55</v>
       </c>
@@ -1298,7 +1599,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A3" s="3" t="s">
         <v>58</v>
       </c>
@@ -1315,7 +1616,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A4" s="3" t="s">
         <v>59</v>
       </c>
@@ -1332,7 +1633,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A5" s="3" t="s">
         <v>61</v>
       </c>
@@ -1349,7 +1650,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A6" s="3" t="s">
         <v>62</v>
       </c>
@@ -1366,7 +1667,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A7" s="3" t="s">
         <v>65</v>
       </c>
@@ -1383,7 +1684,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A8" s="3" t="s">
         <v>66</v>
       </c>
@@ -1400,7 +1701,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A9" s="3" t="s">
         <v>69</v>
       </c>
@@ -1417,7 +1718,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A10" s="3" t="s">
         <v>70</v>
       </c>
@@ -1434,7 +1735,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A11" s="3" t="s">
         <v>71</v>
       </c>
@@ -1451,7 +1752,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>74</v>
       </c>
@@ -1468,7 +1769,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>75</v>
       </c>
@@ -1485,7 +1786,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>76</v>
       </c>
@@ -1502,7 +1803,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>78</v>
       </c>
@@ -1519,7 +1820,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>79</v>
       </c>
@@ -1536,7 +1837,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>83</v>
       </c>
@@ -1553,7 +1854,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A18" s="3" t="s">
         <v>84</v>
       </c>
@@ -1570,7 +1871,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A19" s="3" t="s">
         <v>88</v>
       </c>
@@ -1587,7 +1888,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A20" s="3" t="s">
         <v>90</v>
       </c>
@@ -1604,7 +1905,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A21" s="3" t="s">
         <v>92</v>
       </c>
@@ -1621,7 +1922,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A22" s="3" t="s">
         <v>95</v>
       </c>
@@ -1638,7 +1939,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A23" s="3" t="s">
         <v>97</v>
       </c>
@@ -1655,7 +1956,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A24" s="3" t="s">
         <v>99</v>
       </c>
@@ -1672,7 +1973,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A25" s="3" t="s">
         <v>101</v>
       </c>
@@ -1689,7 +1990,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A26" s="3" t="s">
         <v>102</v>
       </c>
@@ -1706,7 +2007,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A27" s="3" t="s">
         <v>104</v>
       </c>
@@ -1723,7 +2024,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A28" s="3" t="s">
         <v>105</v>
       </c>
@@ -1740,7 +2041,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A29" s="3" t="s">
         <v>106</v>
       </c>
@@ -1757,7 +2058,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A30" s="3" t="s">
         <v>109</v>
       </c>
@@ -1774,7 +2075,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A31" s="3" t="s">
         <v>111</v>
       </c>
@@ -1791,7 +2092,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A32" s="3" t="s">
         <v>106</v>
       </c>
@@ -1808,7 +2109,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A33" s="3" t="s">
         <v>109</v>
       </c>
@@ -1825,7 +2126,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A34" s="3" t="s">
         <v>113</v>
       </c>
@@ -1842,7 +2143,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A35" s="3" t="s">
         <v>115</v>
       </c>
@@ -1859,7 +2160,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A36" s="3" t="s">
         <v>111</v>
       </c>
@@ -1876,7 +2177,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A37" s="3" t="s">
         <v>117</v>
       </c>
@@ -1893,7 +2194,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A38" s="3" t="s">
         <v>119</v>
       </c>
@@ -1910,7 +2211,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A39" s="3" t="s">
         <v>121</v>
       </c>
@@ -1927,7 +2228,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A40" s="3" t="s">
         <v>123</v>
       </c>
@@ -1944,7 +2245,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A41" s="3" t="s">
         <v>125</v>
       </c>
@@ -1961,7 +2262,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A42" s="3" t="s">
         <v>106</v>
       </c>
@@ -1978,7 +2279,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A43" s="3" t="s">
         <v>109</v>
       </c>
@@ -1995,7 +2296,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A44" s="3" t="s">
         <v>111</v>
       </c>
@@ -2012,7 +2313,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A45" s="3" t="s">
         <v>117</v>
       </c>
@@ -2029,7 +2330,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A46" s="3" t="s">
         <v>119</v>
       </c>
@@ -2046,7 +2347,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A47" s="3" t="s">
         <v>113</v>
       </c>
@@ -2063,7 +2364,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A48" s="3" t="s">
         <v>115</v>
       </c>
@@ -2080,7 +2381,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A49" s="3" t="s">
         <v>127</v>
       </c>
@@ -2097,7 +2398,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A50" s="3" t="s">
         <v>129</v>
       </c>
@@ -2114,7 +2415,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A51" s="3" t="s">
         <v>121</v>
       </c>
@@ -2131,7 +2432,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A52" s="3" t="s">
         <v>123</v>
       </c>
@@ -2148,7 +2449,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A53" s="3" t="s">
         <v>125</v>
       </c>
@@ -2165,7 +2466,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A54" s="3" t="s">
         <v>106</v>
       </c>
@@ -2182,7 +2483,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A55" s="3" t="s">
         <v>109</v>
       </c>
@@ -2199,7 +2500,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A56" s="3" t="s">
         <v>111</v>
       </c>
@@ -2216,7 +2517,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A57" s="3" t="s">
         <v>117</v>
       </c>
@@ -2233,7 +2534,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A58" s="3" t="s">
         <v>119</v>
       </c>
@@ -2250,7 +2551,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A59" s="3" t="s">
         <v>113</v>
       </c>
@@ -2267,7 +2568,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A60" s="3" t="s">
         <v>115</v>
       </c>
@@ -2284,7 +2585,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A61" s="3" t="s">
         <v>127</v>
       </c>
@@ -2301,7 +2602,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A62" s="3" t="s">
         <v>129</v>
       </c>
@@ -2318,7 +2619,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A63" s="3" t="s">
         <v>121</v>
       </c>
@@ -2335,7 +2636,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A64" s="3" t="s">
         <v>123</v>
       </c>
@@ -2352,7 +2653,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A65" s="3" t="s">
         <v>125</v>
       </c>
@@ -2369,7 +2670,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A66" s="3" t="s">
         <v>106</v>
       </c>
@@ -2386,7 +2687,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A67" s="3" t="s">
         <v>109</v>
       </c>
@@ -2403,7 +2704,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A68" s="3" t="s">
         <v>111</v>
       </c>
@@ -2420,7 +2721,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A69" s="3" t="s">
         <v>117</v>
       </c>
@@ -2437,7 +2738,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A70" s="3" t="s">
         <v>119</v>
       </c>
@@ -2454,7 +2755,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A71" s="3" t="s">
         <v>131</v>
       </c>
@@ -2471,7 +2772,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A72" s="3" t="s">
         <v>113</v>
       </c>
@@ -2488,7 +2789,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A73" s="3" t="s">
         <v>115</v>
       </c>
@@ -2505,7 +2806,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A74" s="3" t="s">
         <v>127</v>
       </c>
@@ -2522,7 +2823,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A75" s="3" t="s">
         <v>129</v>
       </c>
@@ -2539,7 +2840,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A76" s="3" t="s">
         <v>121</v>
       </c>
@@ -2556,7 +2857,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A77" s="3" t="s">
         <v>123</v>
       </c>
@@ -2573,7 +2874,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="78">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A78" s="3" t="s">
         <v>125</v>
       </c>
@@ -2590,7 +2891,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="79">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A79" s="3" t="s">
         <v>133</v>
       </c>
@@ -2607,7 +2908,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="80">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A80" s="3" t="s">
         <v>106</v>
       </c>
@@ -2624,7 +2925,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="81">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A81" s="3" t="s">
         <v>109</v>
       </c>
@@ -2641,7 +2942,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="82">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A82" s="3" t="s">
         <v>111</v>
       </c>
@@ -2658,7 +2959,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A83" s="3" t="s">
         <v>117</v>
       </c>
@@ -2675,7 +2976,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A84" s="3" t="s">
         <v>119</v>
       </c>
@@ -2692,7 +2993,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A85" s="3" t="s">
         <v>113</v>
       </c>
@@ -2709,7 +3010,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="86">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A86" s="3" t="s">
         <v>115</v>
       </c>
@@ -2726,7 +3027,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A87" s="3" t="s">
         <v>121</v>
       </c>
@@ -2743,7 +3044,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="88">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A88" s="3" t="s">
         <v>123</v>
       </c>
@@ -2760,7 +3061,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="89">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A89" s="3" t="s">
         <v>125</v>
       </c>
@@ -2777,7 +3078,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="90">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A90" s="3" t="s">
         <v>106</v>
       </c>
@@ -2794,7 +3095,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="91">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A91" s="3" t="s">
         <v>109</v>
       </c>
@@ -2811,7 +3112,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="92">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A92" s="3" t="s">
         <v>111</v>
       </c>
@@ -2828,7 +3129,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="93">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A93" s="3" t="s">
         <v>117</v>
       </c>
@@ -2845,7 +3146,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="94">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A94" s="3" t="s">
         <v>119</v>
       </c>
@@ -2862,7 +3163,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="95">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A95" s="3" t="s">
         <v>113</v>
       </c>
@@ -2879,7 +3180,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="96">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A96" s="3" t="s">
         <v>115</v>
       </c>
@@ -2896,7 +3197,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="97">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A97" s="3" t="s">
         <v>127</v>
       </c>
@@ -2913,7 +3214,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="98">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A98" s="3" t="s">
         <v>129</v>
       </c>
@@ -2930,7 +3231,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="99">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A99" s="3" t="s">
         <v>121</v>
       </c>
@@ -2947,7 +3248,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="100">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A100" s="3" t="s">
         <v>123</v>
       </c>
@@ -2964,7 +3265,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="101">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A101" s="3" t="s">
         <v>125</v>
       </c>
@@ -2981,7 +3282,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="102">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A102" s="3" t="s">
         <v>106</v>
       </c>
@@ -2998,7 +3299,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="103">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A103" s="3" t="s">
         <v>109</v>
       </c>
@@ -3015,7 +3316,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="104">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A104" s="3" t="s">
         <v>111</v>
       </c>
@@ -3032,7 +3333,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="105">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A105" s="3" t="s">
         <v>117</v>
       </c>
@@ -3049,7 +3350,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="106">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A106" s="3" t="s">
         <v>119</v>
       </c>
@@ -3066,7 +3367,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="107">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A107" s="3" t="s">
         <v>113</v>
       </c>
@@ -3083,7 +3384,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="108">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A108" s="3" t="s">
         <v>115</v>
       </c>
@@ -3100,7 +3401,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="109">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A109" s="3" t="s">
         <v>127</v>
       </c>
@@ -3117,7 +3418,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="110">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A110" s="3" t="s">
         <v>129</v>
       </c>
@@ -3134,7 +3435,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="111">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A111" s="3" t="s">
         <v>121</v>
       </c>
@@ -3151,7 +3452,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="112">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A112" s="3" t="s">
         <v>123</v>
       </c>
@@ -3168,7 +3469,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="113">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A113" s="3" t="s">
         <v>125</v>
       </c>
@@ -3185,7 +3486,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="114">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A114" s="3" t="s">
         <v>106</v>
       </c>
@@ -3202,7 +3503,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="115">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A115" s="3" t="s">
         <v>109</v>
       </c>
@@ -3219,7 +3520,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="116">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A116" s="3" t="s">
         <v>111</v>
       </c>
@@ -3236,7 +3537,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="117">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A117" s="3" t="s">
         <v>117</v>
       </c>
@@ -3253,7 +3554,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="118">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A118" s="3" t="s">
         <v>119</v>
       </c>
@@ -3270,7 +3571,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="119">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A119" s="3" t="s">
         <v>113</v>
       </c>
@@ -3287,7 +3588,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="120">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A120" s="3" t="s">
         <v>115</v>
       </c>
@@ -3304,7 +3605,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="121">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A121" s="3" t="s">
         <v>127</v>
       </c>
@@ -3321,7 +3622,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="122">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A122" s="3" t="s">
         <v>129</v>
       </c>
@@ -3338,7 +3639,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="123">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A123" s="3" t="s">
         <v>121</v>
       </c>
@@ -3355,7 +3656,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="124">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A124" s="3" t="s">
         <v>123</v>
       </c>
@@ -3372,7 +3673,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="125">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A125" s="3" t="s">
         <v>125</v>
       </c>
@@ -3389,7 +3690,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="126">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A126" s="3" t="s">
         <v>106</v>
       </c>
@@ -3406,7 +3707,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="127">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A127" s="3" t="s">
         <v>109</v>
       </c>
@@ -3423,7 +3724,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="128">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A128" s="3" t="s">
         <v>111</v>
       </c>
@@ -3440,7 +3741,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="129">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A129" s="3" t="s">
         <v>117</v>
       </c>
@@ -3457,7 +3758,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="130">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A130" s="3" t="s">
         <v>119</v>
       </c>
@@ -3474,7 +3775,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="131">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A131" s="3" t="s">
         <v>131</v>
       </c>
@@ -3491,7 +3792,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="132">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A132" s="3" t="s">
         <v>113</v>
       </c>
@@ -3508,7 +3809,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="133">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A133" s="3" t="s">
         <v>115</v>
       </c>
@@ -3525,7 +3826,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="134">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A134" s="3" t="s">
         <v>127</v>
       </c>
@@ -3542,7 +3843,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="135">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A135" s="3" t="s">
         <v>129</v>
       </c>
@@ -3559,7 +3860,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="136">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A136" s="3" t="s">
         <v>121</v>
       </c>
@@ -3576,7 +3877,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="137">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A137" s="3" t="s">
         <v>123</v>
       </c>
@@ -3593,7 +3894,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="138">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A138" s="3" t="s">
         <v>125</v>
       </c>
@@ -3610,7 +3911,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="139">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A139" s="3" t="s">
         <v>106</v>
       </c>
@@ -3627,7 +3928,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="140">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A140" s="3" t="s">
         <v>109</v>
       </c>
@@ -3644,7 +3945,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="141">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A141" s="3" t="s">
         <v>111</v>
       </c>
@@ -3661,7 +3962,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="142">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A142" s="3" t="s">
         <v>117</v>
       </c>
@@ -3678,7 +3979,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="143">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A143" s="3" t="s">
         <v>119</v>
       </c>
@@ -3695,7 +3996,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="144">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A144" s="3" t="s">
         <v>113</v>
       </c>
@@ -3712,7 +4013,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="145">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A145" s="3" t="s">
         <v>115</v>
       </c>
@@ -3729,7 +4030,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="146">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A146" s="3" t="s">
         <v>127</v>
       </c>
@@ -3746,7 +4047,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="147">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A147" s="3" t="s">
         <v>129</v>
       </c>
@@ -3763,7 +4064,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="148">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A148" s="3" t="s">
         <v>121</v>
       </c>
@@ -3780,7 +4081,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="149">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A149" s="3" t="s">
         <v>123</v>
       </c>
@@ -3797,7 +4098,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="150">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A150" s="3" t="s">
         <v>125</v>
       </c>
@@ -3814,7 +4115,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="151">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A151" s="3" t="s">
         <v>106</v>
       </c>
@@ -3831,7 +4132,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="152">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A152" s="3" t="s">
         <v>109</v>
       </c>
@@ -3848,7 +4149,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="153">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A153" s="3" t="s">
         <v>111</v>
       </c>
@@ -3865,7 +4166,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="154">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A154" s="3" t="s">
         <v>117</v>
       </c>
@@ -3882,7 +4183,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="155">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A155" s="3" t="s">
         <v>119</v>
       </c>
@@ -3899,7 +4200,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="156">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A156" s="3" t="s">
         <v>113</v>
       </c>
@@ -3916,7 +4217,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="157">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A157" s="3" t="s">
         <v>115</v>
       </c>
@@ -3933,7 +4234,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="158">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A158" s="3" t="s">
         <v>127</v>
       </c>
@@ -3950,7 +4251,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="159">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A159" s="3" t="s">
         <v>129</v>
       </c>
@@ -3967,7 +4268,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="160">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A160" s="3" t="s">
         <v>121</v>
       </c>
@@ -3984,7 +4285,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="161">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A161" s="3" t="s">
         <v>123</v>
       </c>
@@ -4001,7 +4302,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="162">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A162" s="3" t="s">
         <v>125</v>
       </c>
@@ -4018,7 +4319,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="163">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A163" s="3" t="s">
         <v>106</v>
       </c>
@@ -4035,7 +4336,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="164">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A164" s="3" t="s">
         <v>109</v>
       </c>
@@ -4052,7 +4353,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="165">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A165" s="3" t="s">
         <v>111</v>
       </c>
@@ -4069,7 +4370,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="166">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A166" s="3" t="s">
         <v>117</v>
       </c>
@@ -4086,7 +4387,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="167">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A167" s="3" t="s">
         <v>119</v>
       </c>
@@ -4103,7 +4404,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="168">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A168" s="3" t="s">
         <v>113</v>
       </c>
@@ -4120,7 +4421,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="169">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A169" s="3" t="s">
         <v>115</v>
       </c>
@@ -4137,7 +4438,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="170">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A170" s="3" t="s">
         <v>127</v>
       </c>
@@ -4154,7 +4455,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="171">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A171" s="3" t="s">
         <v>129</v>
       </c>
@@ -4171,7 +4472,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="172">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A172" s="3" t="s">
         <v>121</v>
       </c>
@@ -4188,7 +4489,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="173">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A173" s="3" t="s">
         <v>123</v>
       </c>
@@ -4205,7 +4506,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="174">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A174" s="3" t="s">
         <v>125</v>
       </c>
@@ -4222,7 +4523,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="175">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A175" s="3" t="s">
         <v>135</v>
       </c>
@@ -4239,7 +4540,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="176">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A176" s="3" t="s">
         <v>138</v>
       </c>
@@ -4256,7 +4557,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="177">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A177" s="3" t="s">
         <v>139</v>
       </c>
@@ -4273,7 +4574,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="178">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A178" s="3" t="s">
         <v>140</v>
       </c>
@@ -4290,7 +4591,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="179">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A179" s="3" t="s">
         <v>141</v>
       </c>
@@ -4307,7 +4608,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="180">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A180" s="3" t="s">
         <v>142</v>
       </c>
@@ -4324,7 +4625,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="181">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A181" s="3" t="s">
         <v>143</v>
       </c>
@@ -4341,7 +4642,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="182">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A182" s="3" t="s">
         <v>144</v>
       </c>
@@ -4358,7 +4659,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="183">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A183" s="3" t="s">
         <v>145</v>
       </c>
@@ -4375,7 +4676,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="184">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A184" s="3" t="s">
         <v>146</v>
       </c>
@@ -4394,592 +4695,1610 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="E2"/>
-    <hyperlink r:id="rId2" ref="E3"/>
-    <hyperlink r:id="rId3" ref="E4"/>
-    <hyperlink r:id="rId4" ref="E5"/>
-    <hyperlink r:id="rId5" ref="E6"/>
-    <hyperlink r:id="rId6" ref="E7"/>
-    <hyperlink r:id="rId7" ref="E8"/>
-    <hyperlink r:id="rId8" ref="E9"/>
-    <hyperlink r:id="rId9" ref="E10"/>
-    <hyperlink r:id="rId10" ref="E11"/>
-    <hyperlink r:id="rId11" ref="E12"/>
-    <hyperlink r:id="rId12" ref="E13"/>
-    <hyperlink r:id="rId13" ref="E14"/>
-    <hyperlink r:id="rId14" ref="E15"/>
-    <hyperlink r:id="rId15" ref="E16"/>
-    <hyperlink r:id="rId16" ref="E17"/>
-    <hyperlink r:id="rId17" ref="E18"/>
-    <hyperlink r:id="rId18" ref="E19"/>
-    <hyperlink r:id="rId19" ref="E20"/>
-    <hyperlink r:id="rId20" ref="E21"/>
-    <hyperlink r:id="rId21" ref="E22"/>
-    <hyperlink r:id="rId22" ref="E23"/>
-    <hyperlink r:id="rId23" ref="E24"/>
-    <hyperlink r:id="rId24" ref="E25"/>
-    <hyperlink r:id="rId25" ref="E26"/>
-    <hyperlink r:id="rId26" ref="E27"/>
-    <hyperlink r:id="rId27" ref="E28"/>
-    <hyperlink r:id="rId28" ref="E29"/>
-    <hyperlink r:id="rId29" ref="E30"/>
-    <hyperlink r:id="rId30" ref="E31"/>
-    <hyperlink r:id="rId31" ref="E32"/>
-    <hyperlink r:id="rId32" ref="E33"/>
-    <hyperlink r:id="rId33" ref="E34"/>
-    <hyperlink r:id="rId34" ref="E35"/>
-    <hyperlink r:id="rId35" ref="E36"/>
-    <hyperlink r:id="rId36" ref="E37"/>
-    <hyperlink r:id="rId37" ref="E38"/>
-    <hyperlink r:id="rId38" ref="E39"/>
-    <hyperlink r:id="rId39" ref="E40"/>
-    <hyperlink r:id="rId40" ref="E41"/>
-    <hyperlink r:id="rId41" ref="E42"/>
-    <hyperlink r:id="rId42" ref="E43"/>
-    <hyperlink r:id="rId43" ref="E44"/>
-    <hyperlink r:id="rId44" ref="E45"/>
-    <hyperlink r:id="rId45" ref="E46"/>
-    <hyperlink r:id="rId46" ref="E47"/>
-    <hyperlink r:id="rId47" ref="E48"/>
-    <hyperlink r:id="rId48" ref="E49"/>
-    <hyperlink r:id="rId49" ref="E50"/>
-    <hyperlink r:id="rId50" ref="E51"/>
-    <hyperlink r:id="rId51" ref="E52"/>
-    <hyperlink r:id="rId52" ref="E53"/>
-    <hyperlink r:id="rId53" ref="E54"/>
-    <hyperlink r:id="rId54" ref="E55"/>
-    <hyperlink r:id="rId55" ref="E56"/>
-    <hyperlink r:id="rId56" ref="E57"/>
-    <hyperlink r:id="rId57" ref="E58"/>
-    <hyperlink r:id="rId58" ref="E59"/>
-    <hyperlink r:id="rId59" ref="E60"/>
-    <hyperlink r:id="rId60" ref="E61"/>
-    <hyperlink r:id="rId61" ref="E62"/>
-    <hyperlink r:id="rId62" ref="E63"/>
-    <hyperlink r:id="rId63" ref="E64"/>
-    <hyperlink r:id="rId64" ref="E65"/>
-    <hyperlink r:id="rId65" ref="E66"/>
-    <hyperlink r:id="rId66" ref="E67"/>
-    <hyperlink r:id="rId67" ref="E68"/>
-    <hyperlink r:id="rId68" ref="E69"/>
-    <hyperlink r:id="rId69" ref="E70"/>
-    <hyperlink r:id="rId70" ref="E71"/>
-    <hyperlink r:id="rId71" ref="E72"/>
-    <hyperlink r:id="rId72" ref="E73"/>
-    <hyperlink r:id="rId73" ref="E74"/>
-    <hyperlink r:id="rId74" ref="E75"/>
-    <hyperlink r:id="rId75" ref="E76"/>
-    <hyperlink r:id="rId76" ref="E77"/>
-    <hyperlink r:id="rId77" ref="E78"/>
-    <hyperlink r:id="rId78" ref="E79"/>
-    <hyperlink r:id="rId79" ref="E80"/>
-    <hyperlink r:id="rId80" ref="E81"/>
-    <hyperlink r:id="rId81" ref="E82"/>
-    <hyperlink r:id="rId82" ref="E83"/>
-    <hyperlink r:id="rId83" ref="E84"/>
-    <hyperlink r:id="rId84" ref="E85"/>
-    <hyperlink r:id="rId85" ref="E86"/>
-    <hyperlink r:id="rId86" ref="E87"/>
-    <hyperlink r:id="rId87" ref="E88"/>
-    <hyperlink r:id="rId88" ref="E89"/>
-    <hyperlink r:id="rId89" ref="E90"/>
-    <hyperlink r:id="rId90" ref="E91"/>
-    <hyperlink r:id="rId91" ref="E92"/>
-    <hyperlink r:id="rId92" ref="E93"/>
-    <hyperlink r:id="rId93" ref="E94"/>
-    <hyperlink r:id="rId94" ref="E95"/>
-    <hyperlink r:id="rId95" ref="E96"/>
-    <hyperlink r:id="rId96" ref="E97"/>
-    <hyperlink r:id="rId97" ref="E98"/>
-    <hyperlink r:id="rId98" ref="E99"/>
-    <hyperlink r:id="rId99" ref="E100"/>
-    <hyperlink r:id="rId100" ref="E101"/>
-    <hyperlink r:id="rId101" ref="E102"/>
-    <hyperlink r:id="rId102" ref="E103"/>
-    <hyperlink r:id="rId103" ref="E104"/>
-    <hyperlink r:id="rId104" ref="E105"/>
-    <hyperlink r:id="rId105" ref="E106"/>
-    <hyperlink r:id="rId106" ref="E107"/>
-    <hyperlink r:id="rId107" ref="E108"/>
-    <hyperlink r:id="rId108" ref="E109"/>
-    <hyperlink r:id="rId109" ref="E110"/>
-    <hyperlink r:id="rId110" ref="E111"/>
-    <hyperlink r:id="rId111" ref="E112"/>
-    <hyperlink r:id="rId112" ref="E113"/>
-    <hyperlink r:id="rId113" ref="E114"/>
-    <hyperlink r:id="rId114" ref="E115"/>
-    <hyperlink r:id="rId115" ref="E116"/>
-    <hyperlink r:id="rId116" ref="E117"/>
-    <hyperlink r:id="rId117" ref="E118"/>
-    <hyperlink r:id="rId118" ref="E119"/>
-    <hyperlink r:id="rId119" ref="E120"/>
-    <hyperlink r:id="rId120" ref="E121"/>
-    <hyperlink r:id="rId121" ref="E122"/>
-    <hyperlink r:id="rId122" ref="E123"/>
-    <hyperlink r:id="rId123" ref="E124"/>
-    <hyperlink r:id="rId124" ref="E125"/>
-    <hyperlink r:id="rId125" ref="E126"/>
-    <hyperlink r:id="rId126" ref="E127"/>
-    <hyperlink r:id="rId127" ref="E128"/>
-    <hyperlink r:id="rId128" ref="E129"/>
-    <hyperlink r:id="rId129" ref="E130"/>
-    <hyperlink r:id="rId130" ref="E131"/>
-    <hyperlink r:id="rId131" ref="E132"/>
-    <hyperlink r:id="rId132" ref="E133"/>
-    <hyperlink r:id="rId133" ref="E134"/>
-    <hyperlink r:id="rId134" ref="E135"/>
-    <hyperlink r:id="rId135" ref="E136"/>
-    <hyperlink r:id="rId136" ref="E137"/>
-    <hyperlink r:id="rId137" ref="E138"/>
-    <hyperlink r:id="rId138" ref="E139"/>
-    <hyperlink r:id="rId139" ref="E140"/>
-    <hyperlink r:id="rId140" ref="E141"/>
-    <hyperlink r:id="rId141" ref="E142"/>
-    <hyperlink r:id="rId142" ref="E143"/>
-    <hyperlink r:id="rId143" ref="E144"/>
-    <hyperlink r:id="rId144" ref="E145"/>
-    <hyperlink r:id="rId145" ref="E146"/>
-    <hyperlink r:id="rId146" ref="E147"/>
-    <hyperlink r:id="rId147" ref="E148"/>
-    <hyperlink r:id="rId148" ref="E149"/>
-    <hyperlink r:id="rId149" ref="E150"/>
-    <hyperlink r:id="rId150" ref="E151"/>
-    <hyperlink r:id="rId151" ref="E152"/>
-    <hyperlink r:id="rId152" ref="E153"/>
-    <hyperlink r:id="rId153" ref="E154"/>
-    <hyperlink r:id="rId154" ref="E155"/>
-    <hyperlink r:id="rId155" ref="E156"/>
-    <hyperlink r:id="rId156" ref="E157"/>
-    <hyperlink r:id="rId157" ref="E158"/>
-    <hyperlink r:id="rId158" ref="E159"/>
-    <hyperlink r:id="rId159" ref="E160"/>
-    <hyperlink r:id="rId160" ref="E161"/>
-    <hyperlink r:id="rId161" ref="E162"/>
-    <hyperlink r:id="rId162" ref="E163"/>
-    <hyperlink r:id="rId163" ref="E164"/>
-    <hyperlink r:id="rId164" ref="E165"/>
-    <hyperlink r:id="rId165" ref="E166"/>
-    <hyperlink r:id="rId166" ref="E167"/>
-    <hyperlink r:id="rId167" ref="E168"/>
-    <hyperlink r:id="rId168" ref="E169"/>
-    <hyperlink r:id="rId169" ref="E170"/>
-    <hyperlink r:id="rId170" ref="E171"/>
-    <hyperlink r:id="rId171" ref="E172"/>
-    <hyperlink r:id="rId172" ref="E173"/>
-    <hyperlink r:id="rId173" ref="E174"/>
-    <hyperlink r:id="rId174" ref="E175"/>
-    <hyperlink r:id="rId175" ref="E176"/>
-    <hyperlink r:id="rId176" ref="E177"/>
-    <hyperlink r:id="rId177" ref="E178"/>
-    <hyperlink r:id="rId178" ref="E179"/>
-    <hyperlink r:id="rId179" ref="E180"/>
-    <hyperlink r:id="rId180" ref="E181"/>
-    <hyperlink r:id="rId181" ref="E182"/>
-    <hyperlink r:id="rId182" ref="E183"/>
-    <hyperlink r:id="rId183" ref="E184"/>
+    <hyperlink ref="E2" r:id="rId1"/>
+    <hyperlink ref="E3" r:id="rId2"/>
+    <hyperlink ref="E4" r:id="rId3"/>
+    <hyperlink ref="E5" r:id="rId4"/>
+    <hyperlink ref="E6" r:id="rId5"/>
+    <hyperlink ref="E7" r:id="rId6"/>
+    <hyperlink ref="E8" r:id="rId7"/>
+    <hyperlink ref="E9" r:id="rId8"/>
+    <hyperlink ref="E10" r:id="rId9"/>
+    <hyperlink ref="E11" r:id="rId10"/>
+    <hyperlink ref="E12" r:id="rId11"/>
+    <hyperlink ref="E13" r:id="rId12"/>
+    <hyperlink ref="E14" r:id="rId13"/>
+    <hyperlink ref="E15" r:id="rId14"/>
+    <hyperlink ref="E16" r:id="rId15"/>
+    <hyperlink ref="E17" r:id="rId16"/>
+    <hyperlink ref="E18" r:id="rId17"/>
+    <hyperlink ref="E19" r:id="rId18"/>
+    <hyperlink ref="E20" r:id="rId19"/>
+    <hyperlink ref="E21" r:id="rId20"/>
+    <hyperlink ref="E22" r:id="rId21"/>
+    <hyperlink ref="E23" r:id="rId22"/>
+    <hyperlink ref="E24" r:id="rId23"/>
+    <hyperlink ref="E25" r:id="rId24"/>
+    <hyperlink ref="E26" r:id="rId25"/>
+    <hyperlink ref="E27" r:id="rId26"/>
+    <hyperlink ref="E28" r:id="rId27"/>
+    <hyperlink ref="E29" r:id="rId28"/>
+    <hyperlink ref="E30" r:id="rId29"/>
+    <hyperlink ref="E31" r:id="rId30"/>
+    <hyperlink ref="E32" r:id="rId31"/>
+    <hyperlink ref="E33" r:id="rId32"/>
+    <hyperlink ref="E34" r:id="rId33"/>
+    <hyperlink ref="E35" r:id="rId34"/>
+    <hyperlink ref="E36" r:id="rId35"/>
+    <hyperlink ref="E37" r:id="rId36"/>
+    <hyperlink ref="E38" r:id="rId37"/>
+    <hyperlink ref="E39" r:id="rId38"/>
+    <hyperlink ref="E40" r:id="rId39"/>
+    <hyperlink ref="E41" r:id="rId40"/>
+    <hyperlink ref="E42" r:id="rId41"/>
+    <hyperlink ref="E43" r:id="rId42"/>
+    <hyperlink ref="E44" r:id="rId43"/>
+    <hyperlink ref="E45" r:id="rId44"/>
+    <hyperlink ref="E46" r:id="rId45"/>
+    <hyperlink ref="E47" r:id="rId46"/>
+    <hyperlink ref="E48" r:id="rId47"/>
+    <hyperlink ref="E49" r:id="rId48"/>
+    <hyperlink ref="E50" r:id="rId49"/>
+    <hyperlink ref="E51" r:id="rId50"/>
+    <hyperlink ref="E52" r:id="rId51"/>
+    <hyperlink ref="E53" r:id="rId52"/>
+    <hyperlink ref="E54" r:id="rId53"/>
+    <hyperlink ref="E55" r:id="rId54"/>
+    <hyperlink ref="E56" r:id="rId55"/>
+    <hyperlink ref="E57" r:id="rId56"/>
+    <hyperlink ref="E58" r:id="rId57"/>
+    <hyperlink ref="E59" r:id="rId58"/>
+    <hyperlink ref="E60" r:id="rId59"/>
+    <hyperlink ref="E61" r:id="rId60"/>
+    <hyperlink ref="E62" r:id="rId61"/>
+    <hyperlink ref="E63" r:id="rId62"/>
+    <hyperlink ref="E64" r:id="rId63"/>
+    <hyperlink ref="E65" r:id="rId64"/>
+    <hyperlink ref="E66" r:id="rId65"/>
+    <hyperlink ref="E67" r:id="rId66"/>
+    <hyperlink ref="E68" r:id="rId67"/>
+    <hyperlink ref="E69" r:id="rId68"/>
+    <hyperlink ref="E70" r:id="rId69"/>
+    <hyperlink ref="E71" r:id="rId70"/>
+    <hyperlink ref="E72" r:id="rId71"/>
+    <hyperlink ref="E73" r:id="rId72"/>
+    <hyperlink ref="E74" r:id="rId73"/>
+    <hyperlink ref="E75" r:id="rId74"/>
+    <hyperlink ref="E76" r:id="rId75"/>
+    <hyperlink ref="E77" r:id="rId76"/>
+    <hyperlink ref="E78" r:id="rId77"/>
+    <hyperlink ref="E79" r:id="rId78"/>
+    <hyperlink ref="E80" r:id="rId79"/>
+    <hyperlink ref="E81" r:id="rId80"/>
+    <hyperlink ref="E82" r:id="rId81"/>
+    <hyperlink ref="E83" r:id="rId82"/>
+    <hyperlink ref="E84" r:id="rId83"/>
+    <hyperlink ref="E85" r:id="rId84"/>
+    <hyperlink ref="E86" r:id="rId85"/>
+    <hyperlink ref="E87" r:id="rId86"/>
+    <hyperlink ref="E88" r:id="rId87"/>
+    <hyperlink ref="E89" r:id="rId88"/>
+    <hyperlink ref="E90" r:id="rId89"/>
+    <hyperlink ref="E91" r:id="rId90"/>
+    <hyperlink ref="E92" r:id="rId91"/>
+    <hyperlink ref="E93" r:id="rId92"/>
+    <hyperlink ref="E94" r:id="rId93"/>
+    <hyperlink ref="E95" r:id="rId94"/>
+    <hyperlink ref="E96" r:id="rId95"/>
+    <hyperlink ref="E97" r:id="rId96"/>
+    <hyperlink ref="E98" r:id="rId97"/>
+    <hyperlink ref="E99" r:id="rId98"/>
+    <hyperlink ref="E100" r:id="rId99"/>
+    <hyperlink ref="E101" r:id="rId100"/>
+    <hyperlink ref="E102" r:id="rId101"/>
+    <hyperlink ref="E103" r:id="rId102"/>
+    <hyperlink ref="E104" r:id="rId103"/>
+    <hyperlink ref="E105" r:id="rId104"/>
+    <hyperlink ref="E106" r:id="rId105"/>
+    <hyperlink ref="E107" r:id="rId106"/>
+    <hyperlink ref="E108" r:id="rId107"/>
+    <hyperlink ref="E109" r:id="rId108"/>
+    <hyperlink ref="E110" r:id="rId109"/>
+    <hyperlink ref="E111" r:id="rId110"/>
+    <hyperlink ref="E112" r:id="rId111"/>
+    <hyperlink ref="E113" r:id="rId112"/>
+    <hyperlink ref="E114" r:id="rId113"/>
+    <hyperlink ref="E115" r:id="rId114"/>
+    <hyperlink ref="E116" r:id="rId115"/>
+    <hyperlink ref="E117" r:id="rId116"/>
+    <hyperlink ref="E118" r:id="rId117"/>
+    <hyperlink ref="E119" r:id="rId118"/>
+    <hyperlink ref="E120" r:id="rId119"/>
+    <hyperlink ref="E121" r:id="rId120"/>
+    <hyperlink ref="E122" r:id="rId121"/>
+    <hyperlink ref="E123" r:id="rId122"/>
+    <hyperlink ref="E124" r:id="rId123"/>
+    <hyperlink ref="E125" r:id="rId124"/>
+    <hyperlink ref="E126" r:id="rId125"/>
+    <hyperlink ref="E127" r:id="rId126"/>
+    <hyperlink ref="E128" r:id="rId127"/>
+    <hyperlink ref="E129" r:id="rId128"/>
+    <hyperlink ref="E130" r:id="rId129"/>
+    <hyperlink ref="E131" r:id="rId130"/>
+    <hyperlink ref="E132" r:id="rId131"/>
+    <hyperlink ref="E133" r:id="rId132"/>
+    <hyperlink ref="E134" r:id="rId133"/>
+    <hyperlink ref="E135" r:id="rId134"/>
+    <hyperlink ref="E136" r:id="rId135"/>
+    <hyperlink ref="E137" r:id="rId136"/>
+    <hyperlink ref="E138" r:id="rId137"/>
+    <hyperlink ref="E139" r:id="rId138"/>
+    <hyperlink ref="E140" r:id="rId139"/>
+    <hyperlink ref="E141" r:id="rId140"/>
+    <hyperlink ref="E142" r:id="rId141"/>
+    <hyperlink ref="E143" r:id="rId142"/>
+    <hyperlink ref="E144" r:id="rId143"/>
+    <hyperlink ref="E145" r:id="rId144"/>
+    <hyperlink ref="E146" r:id="rId145"/>
+    <hyperlink ref="E147" r:id="rId146"/>
+    <hyperlink ref="E148" r:id="rId147"/>
+    <hyperlink ref="E149" r:id="rId148"/>
+    <hyperlink ref="E150" r:id="rId149"/>
+    <hyperlink ref="E151" r:id="rId150"/>
+    <hyperlink ref="E152" r:id="rId151"/>
+    <hyperlink ref="E153" r:id="rId152"/>
+    <hyperlink ref="E154" r:id="rId153"/>
+    <hyperlink ref="E155" r:id="rId154"/>
+    <hyperlink ref="E156" r:id="rId155"/>
+    <hyperlink ref="E157" r:id="rId156"/>
+    <hyperlink ref="E158" r:id="rId157"/>
+    <hyperlink ref="E159" r:id="rId158"/>
+    <hyperlink ref="E160" r:id="rId159"/>
+    <hyperlink ref="E161" r:id="rId160"/>
+    <hyperlink ref="E162" r:id="rId161"/>
+    <hyperlink ref="E163" r:id="rId162"/>
+    <hyperlink ref="E164" r:id="rId163"/>
+    <hyperlink ref="E165" r:id="rId164"/>
+    <hyperlink ref="E166" r:id="rId165"/>
+    <hyperlink ref="E167" r:id="rId166"/>
+    <hyperlink ref="E168" r:id="rId167"/>
+    <hyperlink ref="E169" r:id="rId168"/>
+    <hyperlink ref="E170" r:id="rId169"/>
+    <hyperlink ref="E171" r:id="rId170"/>
+    <hyperlink ref="E172" r:id="rId171"/>
+    <hyperlink ref="E173" r:id="rId172"/>
+    <hyperlink ref="E174" r:id="rId173"/>
+    <hyperlink ref="E175" r:id="rId174"/>
+    <hyperlink ref="E176" r:id="rId175"/>
+    <hyperlink ref="E177" r:id="rId176"/>
+    <hyperlink ref="E178" r:id="rId177"/>
+    <hyperlink ref="E179" r:id="rId178"/>
+    <hyperlink ref="E180" r:id="rId179"/>
+    <hyperlink ref="E181" r:id="rId180"/>
+    <hyperlink ref="E182" r:id="rId181"/>
+    <hyperlink ref="E183" r:id="rId182"/>
+    <hyperlink ref="E184" r:id="rId183"/>
   </hyperlinks>
-  <drawing r:id="rId184"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-  <sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I40"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A1" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="D1" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>300</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>301</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>302</v>
+      </c>
+      <c r="I1" s="7"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A2" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B2" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>215</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A3" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>218</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A4" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>220</v>
+      </c>
+      <c r="F4" s="8">
+        <v>0</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A5" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="F5" s="8">
+        <v>0</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A6" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A7" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>227</v>
+      </c>
+      <c r="F7" s="8">
+        <v>0</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A8" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="G8" s="8"/>
+      <c r="H8" s="8" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A9" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="F9" s="8">
+        <v>120</v>
+      </c>
+      <c r="G9" s="8" t="s">
+        <v>232</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A10" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>234</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="G10" s="8"/>
+      <c r="H10" s="8" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A11" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D11" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E11" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="F11" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="G11" s="8"/>
+      <c r="H11" s="8" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A12" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D12" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E12" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="F12" s="8">
+        <v>15</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A13" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D13" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E13" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="F13" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A14" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B14" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C14" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D14" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E14" s="8" t="s">
+        <v>244</v>
+      </c>
+      <c r="F14" s="8">
+        <v>49</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A15" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C15" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E15" s="8" t="s">
+        <v>246</v>
+      </c>
+      <c r="F15" s="8">
+        <v>29</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.15">
+      <c r="A16" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="G16" s="8"/>
+      <c r="H16" s="8" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A17" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B17" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E17" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="F17" s="8">
+        <v>100</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="H17" s="8" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A18" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B18" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E18" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="F18" s="8">
+        <v>4</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="H18" s="8" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A19" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B19" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C19" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E19" s="8" t="s">
+        <v>254</v>
+      </c>
+      <c r="F19" s="8">
+        <v>25</v>
+      </c>
+      <c r="G19" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="H19" s="8" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A20" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B20" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E20" s="8" t="s">
+        <v>256</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="G20" s="8"/>
+      <c r="H20" s="8" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A21" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B21" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C21" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E21" s="8" t="s">
+        <v>259</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="G21" s="8"/>
+      <c r="H21" s="8" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A22" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E22" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="F22" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A23" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E23" s="8" t="s">
+        <v>264</v>
+      </c>
+      <c r="F23" s="8">
+        <v>0</v>
+      </c>
+      <c r="G23" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="H23" s="8" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A24" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E24" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="F24" s="8">
+        <v>0</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="H24" s="8" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A25" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B25" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C25" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E25" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="F25" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A26" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B26" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E26" s="8" t="s">
+        <v>272</v>
+      </c>
+      <c r="F26" s="8">
+        <v>0</v>
+      </c>
+      <c r="G26" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="H26" s="8" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A27" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B27" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C27" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E27" s="8" t="s">
+        <v>274</v>
+      </c>
+      <c r="F27" s="8">
+        <v>52</v>
+      </c>
+      <c r="G27" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="H27" s="8" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A28" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B28" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C28" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E28" s="8" t="s">
+        <v>276</v>
+      </c>
+      <c r="F28" s="8">
+        <v>25.4</v>
+      </c>
+      <c r="G28" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="H28" s="8" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A29" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B29" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C29" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E29" s="8" t="s">
+        <v>278</v>
+      </c>
+      <c r="F29" s="8">
+        <v>23</v>
+      </c>
+      <c r="G29" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="H29" s="8" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A30" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B30" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E30" s="8" t="s">
+        <v>280</v>
+      </c>
+      <c r="F30" s="8">
+        <v>500</v>
+      </c>
+      <c r="G30" s="8" t="s">
+        <v>252</v>
+      </c>
+      <c r="H30" s="8" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A31" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B31" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C31" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>282</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="G31" s="8"/>
+      <c r="H31" s="8" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A32" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B32" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C32" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>284</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="G32" s="8"/>
+      <c r="H32" s="8" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A33" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B33" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C33" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E33" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>262</v>
+      </c>
+      <c r="G33" s="8"/>
+      <c r="H33" s="8" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A34" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B34" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C34" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E34" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="F34" s="8">
+        <v>2.99</v>
+      </c>
+      <c r="G34" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="H34" s="8" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A35" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C35" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E35" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="F35" s="8">
+        <v>0</v>
+      </c>
+      <c r="G35" s="8" t="s">
+        <v>221</v>
+      </c>
+      <c r="H35" s="8" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A36" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B36" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C36" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E36" s="8" t="s">
+        <v>290</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>270</v>
+      </c>
+      <c r="G36" s="8"/>
+      <c r="H36" s="8" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A37" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B37" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C37" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E37" s="8" t="s">
+        <v>292</v>
+      </c>
+      <c r="F37" s="8">
+        <v>21.4</v>
+      </c>
+      <c r="G37" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="H37" s="8" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A38" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B38" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C38" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E38" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>216</v>
+      </c>
+      <c r="G38" s="8"/>
+      <c r="H38" s="8" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A39" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B39" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C39" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E39" s="8" t="s">
+        <v>295</v>
+      </c>
+      <c r="F39" s="8">
+        <v>0</v>
+      </c>
+      <c r="G39" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="H39" s="8" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.15">
+      <c r="A40" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="B40" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C40" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D40" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E40" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="F40" s="8">
+        <v>21</v>
+      </c>
+      <c r="G40" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="H40" s="8" t="s">
+        <v>298</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr enableFormatConditionsCalculation="0">
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:A78"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A1" s="1" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A2" s="3" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A3" s="3" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A4" s="3" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A5" s="3" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A6" s="3" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A7" s="3" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A8" s="3" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A9" s="3" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A10" s="3" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A11" s="3" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A12" s="3" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A13" s="3" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A14" s="3" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A15" s="3" t="s">
         <v>159</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A16" s="3" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A17" s="3" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A18" s="3" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A19" s="3" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A20" s="3" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A21" s="3" t="s">
         <v>164</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A22" s="3" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A23" s="3" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A24" s="3" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A25" s="3" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A26" s="3" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A27" s="3" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A28" s="3" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A29" s="3" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A30" s="3" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A31" s="3" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A32" s="3" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A33" s="3" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A34" s="3" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A35" s="3" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A36" s="3" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A37" s="3" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A38" s="3" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A39" s="3" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A40" s="3" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A41" s="3" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="42">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A42" s="3" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="43">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A43" s="3" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="44">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A44" s="3" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="45">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A45" s="3" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="46">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A46" s="3" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A47" s="3" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="48">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A48" s="3" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="49">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A49" s="3" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="50">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A50" s="3" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="51">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A51" s="3" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="52">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A52" s="3" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="53">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A53" s="3" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="54">
+    <row r="54" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A54" s="3" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="55">
+    <row r="55" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A55" s="3" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="56">
+    <row r="56" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A56" s="3" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A57" s="3" t="s">
         <v>194</v>
       </c>
     </row>
-    <row r="58">
+    <row r="58" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A58" s="3" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="59">
+    <row r="59" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A59" s="3" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="60">
+    <row r="60" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A60" s="3" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="61">
+    <row r="61" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A61" s="3" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="62">
+    <row r="62" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A62" s="3" t="s">
         <v>199</v>
       </c>
     </row>
-    <row r="63">
+    <row r="63" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A63" s="3" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="64">
+    <row r="64" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A64" s="3" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="65">
+    <row r="65" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A65" s="3" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="66">
+    <row r="66" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A66" s="3" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="67">
+    <row r="67" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A67" s="3" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="68">
+    <row r="68" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A68" s="3" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="69">
+    <row r="69" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A69" s="3" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="70">
+    <row r="70" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A70" s="3" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="71">
+    <row r="71" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A71" s="3" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="72">
+    <row r="72" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A72" s="3" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="73">
+    <row r="73" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A73" s="3" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="74">
+    <row r="74" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A74" s="3" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="75">
+    <row r="75" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A75" s="3" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="76">
+    <row r="76" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A76" s="3" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="77">
+    <row r="77" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A77" s="3" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="78">
+    <row r="78" spans="1:1" x14ac:dyDescent="0.15">
       <c r="A78" s="3" t="s">
         <v>213</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>